<commit_message>
Auto update 2026-03-30 16:35:38
</commit_message>
<xml_diff>
--- a/photo_links.xlsx
+++ b/photo_links.xlsx
@@ -2006,7 +2006,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/344/без фоторум\BN-BAG-62-g\001_image_BN-BAG-62-g.png</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/344/без фоторум\BN-BAG-62-g\001_image_BN-BAG-62-g.jpg</t>
         </is>
       </c>
       <c r="E57" t="n">
@@ -4190,7 +4190,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/344/без фоторум\6977703651713\002_image_6977703651713.png</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/344/без фоторум\6977703651713\002_image_6977703651713.jpg</t>
         </is>
       </c>
       <c r="E135" t="n">
@@ -4582,7 +4582,7 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/344/без фоторум\BN-BAG-62-g\002_image_BN-BAG-62-g.png</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/344/без фоторум\BN-BAG-62-g\002_image_BN-BAG-62-g.jpg</t>
         </is>
       </c>
       <c r="E149" t="n">
@@ -6570,7 +6570,7 @@
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/344/без фоторум\6977703651713\3_image_6977703651713.png</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/344/без фоторум\6977703651713\3_image_6977703651713.jpg</t>
         </is>
       </c>
       <c r="E220" t="n">
@@ -6878,7 +6878,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/344/без фоторум\BN-BAG-62-g\3_image_BN-BAG-62-g.png</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/344/без фоторум\BN-BAG-62-g\3_image_BN-BAG-62-g.jpg</t>
         </is>
       </c>
       <c r="E231" t="n">
@@ -10518,7 +10518,7 @@
       </c>
       <c r="D361" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/344/без фоторум\BN-BAG-62-g\5_image_BN-BAG-62-g.png</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/344/без фоторум\BN-BAG-62-g\5_image_BN-BAG-62-g.jpg</t>
         </is>
       </c>
       <c r="E361" t="n">
@@ -12730,7 +12730,7 @@
       </c>
       <c r="D440" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/344/без фоторум\BN-BAG-62-g\6_image_BN-BAG-62-g.png</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/344/без фоторум\BN-BAG-62-g\6_image_BN-BAG-62-g.jpg</t>
         </is>
       </c>
       <c r="E440" t="n">
@@ -14914,7 +14914,7 @@
       </c>
       <c r="D518" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/344/без фоторум\BN-BAG-62-g\7_image_BN-BAG-62-g.png</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/344/без фоторум\BN-BAG-62-g\7_image_BN-BAG-62-g.jpg</t>
         </is>
       </c>
       <c r="E518" t="n">

</xml_diff>